<commit_message>
added WL image to people page
</commit_message>
<xml_diff>
--- a/data/people.xlsx
+++ b/data/people.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jmanning/contextlab.github.io/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B476E088-AC42-4245-89CB-6BC4980731DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC27EA96-6EF7-8443-9C0E-B641AC74417A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="76800" windowHeight="31380" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34560" windowHeight="21660" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="director" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="269">
   <si>
     <t>image</t>
   </si>
@@ -830,6 +830,9 @@
   </si>
   <si>
     <t>alexandra_wingo.png</t>
+  </si>
+  <si>
+    <t>will_lehman.png</t>
   </si>
 </sst>
 </file>
@@ -1558,6 +1561,9 @@
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>268</v>
+      </c>
       <c r="B25" t="s">
         <v>72</v>
       </c>

</xml_diff>

<commit_message>
added JX to people page
</commit_message>
<xml_diff>
--- a/data/people.xlsx
+++ b/data/people.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jmanning/contextlab.github.io/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC27EA96-6EF7-8443-9C0E-B641AC74417A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B8354B1-819F-6E4F-A41D-BD7F81ECD952}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34560" windowHeight="21660" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="18360" yWindow="6560" windowWidth="34560" windowHeight="21660" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="director" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="404" uniqueCount="270">
   <si>
     <t>image</t>
   </si>
@@ -106,9 +106,6 @@
     <t>undergrad</t>
   </si>
   <si>
-    <t>Jennifer is planning to double major in Quantitative Social Science and Comparative Literature. She has a background in mathematics and programming, and is interested in the humanities and literature. She hopes to use machine learning to enhance our understanding of humanitarian issues.</t>
-  </si>
-  <si>
     <t>om_shah.png</t>
   </si>
   <si>
@@ -833,6 +830,12 @@
   </si>
   <si>
     <t>will_lehman.png</t>
+  </si>
+  <si>
+    <t>jennifer_xu.png</t>
+  </si>
+  <si>
+    <t>Jennifer is a Mathematical Data Science major. She is fascinated by understanding how machines "think," whether in biological neural networks or large language models. In her spare time, she enjoys watching videos of tech reviews of mice and keyboards.</t>
   </si>
 </sst>
 </file>
@@ -1317,6 +1320,9 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>268</v>
+      </c>
       <c r="B5" t="s">
         <v>24</v>
       </c>
@@ -1324,254 +1330,254 @@
         <v>25</v>
       </c>
       <c r="E5" t="s">
-        <v>26</v>
+        <v>269</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" t="s">
         <v>27</v>
-      </c>
-      <c r="B6" t="s">
-        <v>28</v>
       </c>
       <c r="D6" t="s">
         <v>25</v>
       </c>
       <c r="E6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" t="s">
         <v>30</v>
-      </c>
-      <c r="B7" t="s">
-        <v>31</v>
       </c>
       <c r="D7" t="s">
         <v>25</v>
       </c>
       <c r="E7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D8" t="s">
         <v>25</v>
       </c>
       <c r="E8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
+        <v>34</v>
+      </c>
+      <c r="B9" t="s">
         <v>35</v>
-      </c>
-      <c r="B9" t="s">
-        <v>36</v>
       </c>
       <c r="D9" t="s">
         <v>25</v>
       </c>
       <c r="E9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D10" t="s">
         <v>25</v>
       </c>
       <c r="E10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D11" t="s">
         <v>25</v>
       </c>
       <c r="E11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
+        <v>41</v>
+      </c>
+      <c r="B12" t="s">
         <v>42</v>
-      </c>
-      <c r="B12" t="s">
-        <v>43</v>
       </c>
       <c r="D12" t="s">
         <v>25</v>
       </c>
       <c r="E12" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>44</v>
+      </c>
+      <c r="B13" t="s">
         <v>45</v>
-      </c>
-      <c r="B13" t="s">
-        <v>46</v>
       </c>
       <c r="D13" t="s">
         <v>25</v>
       </c>
       <c r="E13" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B14" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D14" t="s">
         <v>25</v>
       </c>
       <c r="E14" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B15" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D15" t="s">
         <v>25</v>
       </c>
       <c r="E15" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B16" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D16" t="s">
         <v>25</v>
       </c>
       <c r="E16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
+        <v>53</v>
+      </c>
+      <c r="B17" t="s">
         <v>54</v>
-      </c>
-      <c r="B17" t="s">
-        <v>55</v>
       </c>
       <c r="D17" t="s">
         <v>25</v>
       </c>
       <c r="E17" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
+        <v>56</v>
+      </c>
+      <c r="B18" t="s">
         <v>57</v>
-      </c>
-      <c r="B18" t="s">
-        <v>58</v>
       </c>
       <c r="D18" t="s">
         <v>25</v>
       </c>
       <c r="E18" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D19" t="s">
         <v>25</v>
       </c>
       <c r="E19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B20" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D20" t="s">
         <v>25</v>
       </c>
       <c r="E20" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B21" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D21" t="s">
         <v>25</v>
       </c>
       <c r="E21" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B22" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D22" t="s">
         <v>25</v>
       </c>
       <c r="E22" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B23" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D23" t="s">
         <v>25</v>
       </c>
       <c r="E23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B24" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D24" t="s">
         <v>25</v>
       </c>
       <c r="E24" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B25" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D25" t="s">
         <v>25</v>
       </c>
       <c r="E25" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -1589,31 +1595,31 @@
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B2" t="s">
         <v>75</v>
-      </c>
-      <c r="B2" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B3" t="s">
         <v>77</v>
-      </c>
-      <c r="B3" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B4" t="s">
         <v>79</v>
-      </c>
-      <c r="B4" t="s">
-        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -1631,71 +1637,71 @@
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B2" t="s">
         <v>81</v>
-      </c>
-      <c r="B2" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B3" t="s">
         <v>83</v>
-      </c>
-      <c r="B3" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B4" t="s">
         <v>85</v>
-      </c>
-      <c r="B4" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>87</v>
+      </c>
+      <c r="B6" t="s">
         <v>88</v>
-      </c>
-      <c r="B6" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>89</v>
+      </c>
+      <c r="B7" t="s">
         <v>90</v>
-      </c>
-      <c r="B7" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>91</v>
+      </c>
+      <c r="B8" t="s">
         <v>92</v>
-      </c>
-      <c r="B8" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
+        <v>93</v>
+      </c>
+      <c r="B9" t="s">
         <v>94</v>
-      </c>
-      <c r="B9" t="s">
-        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -1716,61 +1722,61 @@
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>96</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B2" t="s">
         <v>98</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D2" t="s">
         <v>99</v>
       </c>
-      <c r="C2" t="s">
-        <v>84</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>100</v>
-      </c>
-      <c r="E2" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C3" t="s">
+        <v>77</v>
+      </c>
+      <c r="D3" t="s">
         <v>102</v>
       </c>
-      <c r="C3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>103</v>
-      </c>
-      <c r="E3" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C4" t="s">
+        <v>92</v>
+      </c>
+      <c r="D4" t="s">
         <v>105</v>
       </c>
-      <c r="C4" t="s">
-        <v>93</v>
-      </c>
-      <c r="D4" t="s">
-        <v>106</v>
-      </c>
       <c r="E4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -1788,871 +1794,871 @@
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B2" t="s">
         <v>107</v>
-      </c>
-      <c r="B2" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>108</v>
+      </c>
+      <c r="B3" t="s">
         <v>109</v>
-      </c>
-      <c r="B3" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B5" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B10" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B11" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B12" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B13" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B14" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
+        <v>121</v>
+      </c>
+      <c r="B15" t="s">
         <v>122</v>
-      </c>
-      <c r="B15" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
+        <v>123</v>
+      </c>
+      <c r="B16" t="s">
         <v>124</v>
-      </c>
-      <c r="B16" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B17" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B18" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B19" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B20" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B21" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
+        <v>130</v>
+      </c>
+      <c r="B22" t="s">
         <v>131</v>
-      </c>
-      <c r="B22" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B23" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B24" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B25" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B26" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B27" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B28" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B29" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B30" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B31" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B32" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B33" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B34" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B35" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B36" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B37" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B38" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
+        <v>148</v>
+      </c>
+      <c r="B39" t="s">
         <v>149</v>
-      </c>
-      <c r="B39" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
+        <v>150</v>
+      </c>
+      <c r="B40" t="s">
         <v>151</v>
-      </c>
-      <c r="B40" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
+        <v>152</v>
+      </c>
+      <c r="B41" t="s">
         <v>153</v>
-      </c>
-      <c r="B41" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B42" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B43" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B44" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B45" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B46" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B47" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B48" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B49" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B50" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B51" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B52" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B53" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B54" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
+        <v>167</v>
+      </c>
+      <c r="B55" t="s">
         <v>168</v>
-      </c>
-      <c r="B55" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B56" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
+        <v>170</v>
+      </c>
+      <c r="B57" t="s">
         <v>171</v>
-      </c>
-      <c r="B57" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B58" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
+        <v>173</v>
+      </c>
+      <c r="B59" t="s">
         <v>174</v>
-      </c>
-      <c r="B59" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
+        <v>175</v>
+      </c>
+      <c r="B60" t="s">
         <v>176</v>
-      </c>
-      <c r="B60" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B61" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B62" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
+        <v>179</v>
+      </c>
+      <c r="B63" t="s">
         <v>180</v>
-      </c>
-      <c r="B63" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B64" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B65" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B66" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B67" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B68" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B69" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B70" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B71" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B72" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B73" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B74" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B75" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
+        <v>193</v>
+      </c>
+      <c r="B76" t="s">
         <v>194</v>
-      </c>
-      <c r="B76" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B77" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B78" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B79" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B80" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B81" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
+        <v>200</v>
+      </c>
+      <c r="B82" t="s">
         <v>201</v>
-      </c>
-      <c r="B82" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
+        <v>202</v>
+      </c>
+      <c r="B83" t="s">
         <v>203</v>
-      </c>
-      <c r="B83" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B84" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B85" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B86" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B87" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B88" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B89" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B90" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B91" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B92" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B93" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
+        <v>214</v>
+      </c>
+      <c r="B94" t="s">
         <v>215</v>
-      </c>
-      <c r="B94" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B95" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B96" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
+        <v>218</v>
+      </c>
+      <c r="B97" t="s">
         <v>219</v>
-      </c>
-      <c r="B97" t="s">
-        <v>220</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B98" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B99" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B100" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B101" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B102" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B103" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B104" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B105" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B106" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B107" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B108" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B109" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -2670,131 +2676,131 @@
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>233</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>234</v>
+      </c>
+      <c r="B2" t="s">
         <v>235</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>236</v>
-      </c>
-      <c r="C2" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B3" t="s">
+        <v>237</v>
+      </c>
+      <c r="C3" t="s">
         <v>238</v>
-      </c>
-      <c r="C3" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>239</v>
+      </c>
+      <c r="B4" t="s">
         <v>240</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>241</v>
-      </c>
-      <c r="C4" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
+        <v>242</v>
+      </c>
+      <c r="B5" t="s">
         <v>243</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>244</v>
-      </c>
-      <c r="C5" t="s">
-        <v>245</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>245</v>
+      </c>
+      <c r="B6" t="s">
         <v>246</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>247</v>
-      </c>
-      <c r="C6" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>248</v>
+      </c>
+      <c r="B7" t="s">
         <v>249</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>250</v>
-      </c>
-      <c r="C7" t="s">
-        <v>251</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>251</v>
+      </c>
+      <c r="B8" t="s">
         <v>252</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>253</v>
-      </c>
-      <c r="C8" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
+        <v>254</v>
+      </c>
+      <c r="B9" t="s">
         <v>255</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>256</v>
-      </c>
-      <c r="C9" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
+        <v>257</v>
+      </c>
+      <c r="B10" t="s">
         <v>258</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>259</v>
-      </c>
-      <c r="C10" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
+        <v>260</v>
+      </c>
+      <c r="B11" t="s">
         <v>261</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>262</v>
-      </c>
-      <c r="C11" t="s">
-        <v>263</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
+        <v>263</v>
+      </c>
+      <c r="B12" t="s">
         <v>264</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>265</v>
-      </c>
-      <c r="C12" t="s">
-        <v>266</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added AM image + updated bio to people page
</commit_message>
<xml_diff>
--- a/data/people.xlsx
+++ b/data/people.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jmanning/contextlab.github.io/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B8354B1-819F-6E4F-A41D-BD7F81ECD952}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFD6C5A0-32C7-CE44-9158-76A16B6220F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="18360" yWindow="6560" windowWidth="34560" windowHeight="21660" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="35720" yWindow="8360" windowWidth="34560" windowHeight="21660" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="director" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="404" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="271">
   <si>
     <t>image</t>
   </si>
@@ -142,9 +142,6 @@
     <t>aidan miller</t>
   </si>
   <si>
-    <t>Aidan is a pre-med student interested in how we can learn as quickly and efficiently as possible. He is a dedicated practitioner of memory "hacks" like the chaine method, story method, and method of loci.</t>
-  </si>
-  <si>
     <t>alexandra wingo</t>
   </si>
   <si>
@@ -836,6 +833,12 @@
   </si>
   <si>
     <t>Jennifer is a Mathematical Data Science major. She is fascinated by understanding how machines "think," whether in biological neural networks or large language models. In her spare time, she enjoys watching videos of tech reviews of mice and keyboards.</t>
+  </si>
+  <si>
+    <t>aidan_miller.png</t>
+  </si>
+  <si>
+    <t>Aidan Miller is a pre-med student at Dartmouth College, majoring in Biology, minor in Spanish, and graduating in 2028. He joined the Contextual Dynamics Lab in fall 2025, where his interests center on advanced learning and memory techniques, including the method of loci and PAO systems.</t>
   </si>
 </sst>
 </file>
@@ -1321,7 +1324,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B5" t="s">
         <v>24</v>
@@ -1330,7 +1333,7 @@
         <v>25</v>
       </c>
       <c r="E5" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -1387,6 +1390,9 @@
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>269</v>
+      </c>
       <c r="B10" t="s">
         <v>37</v>
       </c>
@@ -1394,190 +1400,190 @@
         <v>25</v>
       </c>
       <c r="E10" t="s">
-        <v>38</v>
+        <v>270</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D11" t="s">
         <v>25</v>
       </c>
       <c r="E11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
+        <v>40</v>
+      </c>
+      <c r="B12" t="s">
         <v>41</v>
-      </c>
-      <c r="B12" t="s">
-        <v>42</v>
       </c>
       <c r="D12" t="s">
         <v>25</v>
       </c>
       <c r="E12" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B13" t="s">
         <v>44</v>
-      </c>
-      <c r="B13" t="s">
-        <v>45</v>
       </c>
       <c r="D13" t="s">
         <v>25</v>
       </c>
       <c r="E13" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B14" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D14" t="s">
         <v>25</v>
       </c>
       <c r="E14" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B15" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D15" t="s">
         <v>25</v>
       </c>
       <c r="E15" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D16" t="s">
         <v>25</v>
       </c>
       <c r="E16" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B17" t="s">
         <v>53</v>
-      </c>
-      <c r="B17" t="s">
-        <v>54</v>
       </c>
       <c r="D17" t="s">
         <v>25</v>
       </c>
       <c r="E17" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
+        <v>55</v>
+      </c>
+      <c r="B18" t="s">
         <v>56</v>
-      </c>
-      <c r="B18" t="s">
-        <v>57</v>
       </c>
       <c r="D18" t="s">
         <v>25</v>
       </c>
       <c r="E18" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D19" t="s">
         <v>25</v>
       </c>
       <c r="E19" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B20" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D20" t="s">
         <v>25</v>
       </c>
       <c r="E20" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B21" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D21" t="s">
         <v>25</v>
       </c>
       <c r="E21" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B22" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D22" t="s">
         <v>25</v>
       </c>
       <c r="E22" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B23" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D23" t="s">
         <v>25</v>
       </c>
       <c r="E23" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B24" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D24" t="s">
         <v>25</v>
       </c>
       <c r="E24" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B25" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D25" t="s">
         <v>25</v>
       </c>
       <c r="E25" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -1595,31 +1601,31 @@
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B2" t="s">
         <v>74</v>
-      </c>
-      <c r="B2" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B3" t="s">
         <v>76</v>
-      </c>
-      <c r="B3" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>77</v>
+      </c>
+      <c r="B4" t="s">
         <v>78</v>
-      </c>
-      <c r="B4" t="s">
-        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -1637,71 +1643,71 @@
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B2" t="s">
         <v>80</v>
-      </c>
-      <c r="B2" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B3" t="s">
         <v>82</v>
-      </c>
-      <c r="B3" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B4" t="s">
         <v>84</v>
-      </c>
-      <c r="B4" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B6" t="s">
         <v>87</v>
-      </c>
-      <c r="B6" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B7" t="s">
         <v>89</v>
-      </c>
-      <c r="B7" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B8" t="s">
         <v>91</v>
-      </c>
-      <c r="B8" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
+        <v>92</v>
+      </c>
+      <c r="B9" t="s">
         <v>93</v>
-      </c>
-      <c r="B9" t="s">
-        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -1722,61 +1728,61 @@
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>95</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B2" t="s">
         <v>97</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D2" t="s">
         <v>98</v>
       </c>
-      <c r="C2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>99</v>
-      </c>
-      <c r="E2" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C3" t="s">
+        <v>76</v>
+      </c>
+      <c r="D3" t="s">
         <v>101</v>
       </c>
-      <c r="C3" t="s">
-        <v>77</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>102</v>
-      </c>
-      <c r="E3" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B4" t="s">
+        <v>103</v>
+      </c>
+      <c r="C4" t="s">
+        <v>91</v>
+      </c>
+      <c r="D4" t="s">
         <v>104</v>
       </c>
-      <c r="C4" t="s">
-        <v>92</v>
-      </c>
-      <c r="D4" t="s">
-        <v>105</v>
-      </c>
       <c r="E4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -1794,871 +1800,871 @@
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B2" t="s">
         <v>106</v>
-      </c>
-      <c r="B2" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>107</v>
+      </c>
+      <c r="B3" t="s">
         <v>108</v>
-      </c>
-      <c r="B3" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B10" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B11" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B12" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B13" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B14" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
+        <v>120</v>
+      </c>
+      <c r="B15" t="s">
         <v>121</v>
-      </c>
-      <c r="B15" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
+        <v>122</v>
+      </c>
+      <c r="B16" t="s">
         <v>123</v>
-      </c>
-      <c r="B16" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B17" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B18" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B19" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B20" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B21" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
+        <v>129</v>
+      </c>
+      <c r="B22" t="s">
         <v>130</v>
-      </c>
-      <c r="B22" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B23" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B24" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B25" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B26" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B27" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B28" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B29" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B30" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B31" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B32" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B33" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B34" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B35" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B36" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B37" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B38" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
+        <v>147</v>
+      </c>
+      <c r="B39" t="s">
         <v>148</v>
-      </c>
-      <c r="B39" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
+        <v>149</v>
+      </c>
+      <c r="B40" t="s">
         <v>150</v>
-      </c>
-      <c r="B40" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
+        <v>151</v>
+      </c>
+      <c r="B41" t="s">
         <v>152</v>
-      </c>
-      <c r="B41" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B42" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B43" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B44" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B45" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B46" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B47" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B48" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B49" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B50" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B51" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B52" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B53" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B54" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
+        <v>166</v>
+      </c>
+      <c r="B55" t="s">
         <v>167</v>
-      </c>
-      <c r="B55" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B56" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
+        <v>169</v>
+      </c>
+      <c r="B57" t="s">
         <v>170</v>
-      </c>
-      <c r="B57" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B58" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
+        <v>172</v>
+      </c>
+      <c r="B59" t="s">
         <v>173</v>
-      </c>
-      <c r="B59" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
+        <v>174</v>
+      </c>
+      <c r="B60" t="s">
         <v>175</v>
-      </c>
-      <c r="B60" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B61" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B62" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
+        <v>178</v>
+      </c>
+      <c r="B63" t="s">
         <v>179</v>
-      </c>
-      <c r="B63" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B64" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B65" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B66" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B67" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B68" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B69" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B70" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B71" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B72" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B73" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B74" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B75" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
+        <v>192</v>
+      </c>
+      <c r="B76" t="s">
         <v>193</v>
-      </c>
-      <c r="B76" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B77" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B78" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B79" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B80" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B81" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
+        <v>199</v>
+      </c>
+      <c r="B82" t="s">
         <v>200</v>
-      </c>
-      <c r="B82" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
+        <v>201</v>
+      </c>
+      <c r="B83" t="s">
         <v>202</v>
-      </c>
-      <c r="B83" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B84" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B85" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B86" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B87" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B88" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B89" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B90" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B91" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B92" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B93" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
+        <v>213</v>
+      </c>
+      <c r="B94" t="s">
         <v>214</v>
-      </c>
-      <c r="B94" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B95" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B96" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
+        <v>217</v>
+      </c>
+      <c r="B97" t="s">
         <v>218</v>
-      </c>
-      <c r="B97" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B98" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B99" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B100" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B101" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B102" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B103" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B104" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B105" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B106" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B107" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B108" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B109" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -2676,131 +2682,131 @@
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>232</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>233</v>
+      </c>
+      <c r="B2" t="s">
         <v>234</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>235</v>
-      </c>
-      <c r="C2" t="s">
-        <v>236</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B3" t="s">
+        <v>236</v>
+      </c>
+      <c r="C3" t="s">
         <v>237</v>
-      </c>
-      <c r="C3" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>238</v>
+      </c>
+      <c r="B4" t="s">
         <v>239</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>240</v>
-      </c>
-      <c r="C4" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
+        <v>241</v>
+      </c>
+      <c r="B5" t="s">
         <v>242</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>243</v>
-      </c>
-      <c r="C5" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>244</v>
+      </c>
+      <c r="B6" t="s">
         <v>245</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>246</v>
-      </c>
-      <c r="C6" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>247</v>
+      </c>
+      <c r="B7" t="s">
         <v>248</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>249</v>
-      </c>
-      <c r="C7" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>250</v>
+      </c>
+      <c r="B8" t="s">
         <v>251</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>252</v>
-      </c>
-      <c r="C8" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
+        <v>253</v>
+      </c>
+      <c r="B9" t="s">
         <v>254</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>255</v>
-      </c>
-      <c r="C9" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
+        <v>256</v>
+      </c>
+      <c r="B10" t="s">
         <v>257</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>258</v>
-      </c>
-      <c r="C10" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
+        <v>259</v>
+      </c>
+      <c r="B11" t="s">
         <v>260</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>261</v>
-      </c>
-      <c r="C11" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
+        <v>262</v>
+      </c>
+      <c r="B12" t="s">
         <v>263</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>264</v>
-      </c>
-      <c r="C12" t="s">
-        <v>265</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
style tweaks to AM bio
</commit_message>
<xml_diff>
--- a/data/people.xlsx
+++ b/data/people.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jmanning/contextlab.github.io/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFD6C5A0-32C7-CE44-9158-76A16B6220F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF52BB1A-7E8F-8941-B899-5A12E1200371}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="35720" yWindow="8360" windowWidth="34560" windowHeight="21660" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -838,7 +838,7 @@
     <t>aidan_miller.png</t>
   </si>
   <si>
-    <t>Aidan Miller is a pre-med student at Dartmouth College, majoring in Biology, minor in Spanish, and graduating in 2028. He joined the Contextual Dynamics Lab in fall 2025, where his interests center on advanced learning and memory techniques, including the method of loci and PAO systems.</t>
+    <t>Aidan is a pre-med student at Dartmouth College, majoring in Biology, minor in Spanish, and graduating in 2028. He joined the Contextual Dynamics Lab in fall 2025, where his interests center on advanced learning and memory techniques, including the method of loci and PAO systems.</t>
   </si>
 </sst>
 </file>
@@ -857,6 +857,7 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">

</xml_diff>

<commit_message>
fix: preserve existing bio when using --skip-llm
Added get_existing_bio() to check spreadsheet before generating fallback bio.
Now --skip-llm will use existing bio from spreadsheet if available.
</commit_message>
<xml_diff>
--- a/data/people.xlsx
+++ b/data/people.xlsx
@@ -520,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -955,6 +955,28 @@
       <c r="E20" t="inlineStr">
         <is>
           <t>Will is a '27 from Salt Lake City, Utah. He likes skiing, playing hockey, and working on new projects.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>theo_larson.png</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>theo larson</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>undergrad</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Theo is a '29 from Brooklyn, New York and a prospective major in Economics and History. In his free time, he enjoys reading, playing board games, and taking walks with his dog Sunny.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
shorten position text for Kirsten and Lucy
</commit_message>
<xml_diff>
--- a/data/people.xlsx
+++ b/data/people.xlsx
@@ -1179,7 +1179,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Lecturer at Princeton University</t>
+          <t>Princeton University</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1201,7 +1201,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Assistant Professor at University of Montana</t>
+          <t>University of Montana</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">

</xml_diff>

<commit_message>
fix alumni ordering: reverse chronological (recent first)
- Sorted alumni_undergrads in spreadsheet by year descending
- Fixed offboard_member.py to insert at top of alumni list instead of appending
</commit_message>
<xml_diff>
--- a/data/people.xlsx
+++ b/data/people.xlsx
@@ -1390,103 +1390,103 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Rodrigo Vega Ayllon</t>
+          <t>Chelsea Joe</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Miel Wewerka</t>
+          <t>Annabelle Morrow</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Manraaj Singh</t>
+          <t>Jackson C. Sandrich</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2026</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Can Kam</t>
+          <t>Luca Gandrud</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2026</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Rohan Goyal</t>
+          <t>Owen Phillips</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2026</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Harrison Stropkay</t>
+          <t>Rodrigo Vega Ayllon</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2024-2025</t>
+          <t>2025</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Abigayle McCusker</t>
+          <t>Harrison Stropkay</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024-2025</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Torsha Chakraverty</t>
+          <t>Jake McDermid</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2023-2025</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Chloe Terestchenko</t>
+          <t>Miel Wewerka</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1498,7 +1498,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Ansh Motiani</t>
+          <t>Manraaj Singh</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1510,7 +1510,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Kaitlyn Peng</t>
+          <t>Can Kam</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1522,7 +1522,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Everett Tai</t>
+          <t>Rohan Goyal</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1534,7 +1534,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Andrew Cao</t>
+          <t>Abigayle McCusker</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1546,79 +1546,79 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Michael Chen</t>
+          <t>Torsha Chakraverty</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2024</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Jake McDermid</t>
+          <t>Chloe Terestchenko</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2023-2025</t>
+          <t>2024</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Grady Redding</t>
+          <t>Ansh Motiani</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2024</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>DJ Matusz</t>
+          <t>Kaitlyn Peng</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2024</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Aaryan Agarwal</t>
+          <t>Everett Tai</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2024</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Maura Hough</t>
+          <t>Andrew Cao</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2024</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Emma Reeder</t>
+          <t>Michael Chen</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1630,55 +1630,55 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Safwan Rashid</t>
+          <t>Grady Redding</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023-2024</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Francisca Fadairo</t>
+          <t>DJ Matusz</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023-2024</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ameer Talha Yasser</t>
+          <t>Aaryan Agarwal</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023-2024</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Yue Zhuo</t>
+          <t>Maura Hough</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023-2024</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Megan Liu</t>
+          <t>Emma Reeder</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1690,67 +1690,67 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Charles Baker</t>
+          <t>Megan Liu</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023-2024</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Andrew Shi</t>
+          <t>Mira Chiruvolu</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023-2024</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Ash Chinta</t>
+          <t>Ansh Patel</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022-2024</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Xueyao Zheng</t>
+          <t>Kunal Jha</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2021-2024</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Sergio Campos Legonia</t>
+          <t>Daniel Carstensen</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2021-2024</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Elias Emery</t>
+          <t>Safwan Rashid</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1762,7 +1762,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Yvonne Chen</t>
+          <t>Francisca Fadairo</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1774,7 +1774,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>William McCall</t>
+          <t>Ameer Talha Yasser</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1786,7 +1786,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Natalie Schreder</t>
+          <t>Yue Zhuo</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1798,7 +1798,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Raselas Dessalegn</t>
+          <t>Charles Baker</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1810,7 +1810,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Grace Wang</t>
+          <t>Andrew Shi</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1822,127 +1822,127 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Mira Chiruvolu</t>
+          <t>Ash Chinta</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Anna Mikhailova</t>
+          <t>Xueyao Zheng</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Ansh Patel</t>
+          <t>Sergio Campos Legonia</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2022-2024</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Ziyan Zhu</t>
+          <t>Elias Emery</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2022-2023</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Benjamin Lehrburger</t>
+          <t>Yvonne Chen</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Thomas Corrado</t>
+          <t>William McCall</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Samuel Crombie</t>
+          <t>Natalie Schreder</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Alexander Marcoux</t>
+          <t>Raselas Dessalegn</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Jessna Brar</t>
+          <t>Grace Wang</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Wenhua Liang</t>
+          <t>Ziyan Zhu</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022-2023</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Kevin Cao</t>
+          <t>Anna Mikhailova</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1954,7 +1954,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Goutham Veeramachaneni</t>
+          <t>Benjamin Lehrburger</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1966,7 +1966,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Zachary Somma</t>
+          <t>Thomas Corrado</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1978,7 +1978,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Dawson Haddox</t>
+          <t>Samuel Crombie</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1990,7 +1990,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Swestha Jain</t>
+          <t>Alexander Marcoux</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2002,175 +2002,175 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Aidan Adams</t>
+          <t>Jessna Brar</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2022</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Damini Kohli</t>
+          <t>Wenhua Liang</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2022</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Kunal Jha</t>
+          <t>Kevin Cao</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2021-2024</t>
+          <t>2022</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Daniel Carstensen</t>
+          <t>Goutham Veeramachaneni</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2021-2024</t>
+          <t>2022</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Brian Chiang</t>
+          <t>Zachary Somma</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2021-2022</t>
+          <t>2022</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Daniel Ha</t>
+          <t>Dawson Haddox</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2022</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Darren Gu</t>
+          <t>Swestha Jain</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2020-2021</t>
+          <t>2022</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Tyler Chen</t>
+          <t>Brian Chiang</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2020-2022</t>
+          <t>2021-2022</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Tehut Biru</t>
+          <t>Tyler Chen</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2020-2021</t>
+          <t>2020-2022</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Chris Suh</t>
+          <t>Chris Jun</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2020-2021</t>
+          <t>2020-2022</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Helen Liu</t>
+          <t>Ethan Adner</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2020-2022</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Kelly Rutherford</t>
+          <t>Aidan Adams</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2021</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Chris Jun</t>
+          <t>Damini Kohli</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2020-2022</t>
+          <t>2021</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Ethan Adner</t>
+          <t>Daniel Ha</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2020-2022</t>
+          <t>2021</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Chris Long</t>
+          <t>Darren Gu</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2182,7 +2182,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Esme Chen</t>
+          <t>Tehut Biru</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2194,55 +2194,55 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Luca Lit</t>
+          <t>Chris Suh</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2020-2021</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Vivian Tran</t>
+          <t>Chris Long</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2020-2021</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Greg Han</t>
+          <t>Esme Chen</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2020-2021</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Austin Zhang</t>
+          <t>Tudor Muntianu</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2019-2021</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Chelsea Uddenberg</t>
+          <t>Helen Liu</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2254,7 +2254,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Shane Hewitt</t>
+          <t>Kelly Rutherford</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2266,7 +2266,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Chetan Palvuluri</t>
+          <t>Luca Lit</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2278,379 +2278,379 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Aaron Lee</t>
+          <t>Vivian Tran</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2019-2020</t>
+          <t>2020</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Anne George</t>
+          <t>Greg Han</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2019-2020</t>
+          <t>2020</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Sarah Park</t>
+          <t>Austin Zhang</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2019-2020</t>
+          <t>2020</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Shane Park</t>
+          <t>Chelsea Uddenberg</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2019-2020</t>
+          <t>2020</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>William Chen</t>
+          <t>Shane Hewitt</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2019-2020</t>
+          <t>2020</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Tudor Muntianu</t>
+          <t>Chetan Palvuluri</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2019-2021</t>
+          <t>2020</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>William Baxley</t>
+          <t>Aaron Lee</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2018-2019</t>
+          <t>2019-2020</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Ann Carpenter</t>
+          <t>Anne George</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2019-2020</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Seung Ju Lee</t>
+          <t>Sarah Park</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2019-2020</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Mustafa Nasir-Moin</t>
+          <t>Shane Park</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2019-2020</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Iain Sheerin</t>
+          <t>William Chen</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2019-2020</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Darya Romanova</t>
+          <t>Alejandro Martinez</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2018-2020</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Alejandro Martinez</t>
+          <t>Madeline Lee</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2018-2020</t>
+          <t>2016-2020</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Rachael Chacko</t>
+          <t>William Baxley</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2018-2019</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Kirsten Soh</t>
+          <t>Paxton Fitzpatrick</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2017-2019</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Paxton Fitzpatrick</t>
+          <t>Ann Carpenter</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2017-2019</t>
+          <t>2018</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Stephen Satterthwaite</t>
+          <t>Seung Ju Lee</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2017-2018</t>
+          <t>2018</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Bryan Bollinger</t>
+          <t>Mustafa Nasir-Moin</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2017-2018</t>
+          <t>2018</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Christina Lu</t>
+          <t>Iain Sheerin</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2018</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Armando Oritz</t>
+          <t>Darya Romanova</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2018</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Campbell Field</t>
+          <t>Rachael Chacko</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2016-2018</t>
+          <t>2018</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Madeline Lee</t>
+          <t>Kirsten Soh</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2016-2020</t>
+          <t>2018</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Wei Liang Samuel Ching</t>
+          <t>Stephen Satterthwaite</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2016-2017</t>
+          <t>2017-2018</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Marisol Tracy</t>
+          <t>Bryan Bollinger</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2016-2017</t>
+          <t>2017-2018</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Allison Frantz</t>
+          <t>Campbell Field</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2016-2017</t>
+          <t>2016-2018</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Aamuktha Porika</t>
+          <t>Christina Lu</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2016-2017</t>
+          <t>2017</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Jake Rost</t>
+          <t>Armando Oritz</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>2017</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Clara Silvanic</t>
+          <t>Wei Liang Samuel Ching</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>2016-2017</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Aman Agarwal</t>
+          <t>Marisol Tracy</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>2016-2017</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Joseph Finkelstein</t>
+          <t>Allison Frantz</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>2016-2017</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Sheherzad Mohydin</t>
+          <t>Aamuktha Porika</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>2016-2017</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Peter Tran</t>
+          <t>Jake Rost</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -2662,7 +2662,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Gal Perlman</t>
+          <t>Clara Silvanic</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -2674,7 +2674,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Jessica Tin</t>
+          <t>Aman Agarwal</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -2686,60 +2686,60 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Chelsea Joe</t>
+          <t>Joseph Finkelstein</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2016</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Annabelle Morrow</t>
+          <t>Sheherzad Mohydin</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2016</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Jackson C. Sandrich</t>
+          <t>Peter Tran</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2016</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Luca Gandrud</t>
+          <t>Gal Perlman</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2016</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Owen Phillips</t>
+          <t>Jessica Tin</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2016</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix alumni date ranges and offboarding script
- Fixed dates for 5 undergrad alumni to show full range (start-end):
  Chelsea Joe (2024-2026), Annabelle Morrow (2025-2026),
  Jackson C. Sandrich (2025-2026), Luca Gandrud (2025-2026),
  Owen Phillips (2025-2026)
- Updated offboard_member.py to extract start year from CV and
  store full date range in alumni sheet instead of just end year

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/people.xlsx
+++ b/data/people.xlsx
@@ -825,6 +825,11 @@
       </c>
     </row>
     <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>azaire_andre.png</t>
+        </is>
+      </c>
       <c r="B14" t="inlineStr">
         <is>
           <t>azaire andre</t>
@@ -837,7 +842,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Azaire is a Mathematics and Anthropology double major. She is particularly interested in understanding complex systems like brain networks and financial markets.</t>
+          <t>Azaire is a Dartmouth student studying mathematics and anthropology, with interests in health equity, education, and community leadership. She enjoys swimming and cheering, and is actively involved in campus organizations that support mentorship and inclusion.</t>
         </is>
       </c>
     </row>
@@ -1395,7 +1400,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2024-2026</t>
         </is>
       </c>
     </row>
@@ -1407,7 +1412,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025-2026</t>
         </is>
       </c>
     </row>
@@ -1419,7 +1424,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025-2026</t>
         </is>
       </c>
     </row>
@@ -1431,7 +1436,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025-2026</t>
         </is>
       </c>
     </row>
@@ -1443,7 +1448,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025-2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix alumni ordering: use CV order within same start year
- Changed secondary sort from alphabetical to stable (preserves spreadsheet order)
- Reordered spreadsheet to match CV order (by CV entry number descending)
- 2025 starters now correctly ordered: Jackson, Luca, Annabelle, Owen, Rodrigo

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/people.xlsx
+++ b/data/people.xlsx
@@ -1395,19 +1395,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Chelsea Joe</t>
+          <t>Jackson C. Sandrich</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2024-2026</t>
+          <t>2025-2026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Annabelle Morrow</t>
+          <t>Luca Gandrud</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1419,7 +1419,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Jackson C. Sandrich</t>
+          <t>Annabelle Morrow</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1431,7 +1431,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Luca Gandrud</t>
+          <t>Owen Phillips</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1443,24 +1443,24 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Owen Phillips</t>
+          <t>Rodrigo Vega Ayllon</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2025</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Rodrigo Vega Ayllon</t>
+          <t>Chelsea Joe</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024-2026</t>
         </is>
       </c>
     </row>
@@ -1479,19 +1479,19 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Jake McDermid</t>
+          <t>Miel Wewerka</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2023-2025</t>
+          <t>2024</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Miel Wewerka</t>
+          <t>Manraaj Singh</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1503,7 +1503,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Manraaj Singh</t>
+          <t>Can Kam</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1515,7 +1515,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Can Kam</t>
+          <t>Rohan Goyal</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1527,7 +1527,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Rohan Goyal</t>
+          <t>Abigayle McCusker</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1539,7 +1539,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Abigayle McCusker</t>
+          <t>Torsha Chakraverty</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1551,7 +1551,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Torsha Chakraverty</t>
+          <t>Chloe Terestchenko</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1563,7 +1563,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Chloe Terestchenko</t>
+          <t>Ansh Motiani</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1575,7 +1575,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Ansh Motiani</t>
+          <t>Kaitlyn Peng</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1587,7 +1587,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Kaitlyn Peng</t>
+          <t>Everett Tai</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1599,7 +1599,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Everett Tai</t>
+          <t>Andrew Cao</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1611,12 +1611,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Andrew Cao</t>
+          <t>Jake McDermid</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2023-2025</t>
         </is>
       </c>
     </row>
@@ -1719,43 +1719,43 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Ansh Patel</t>
+          <t>Safwan Rashid</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2022-2024</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Kunal Jha</t>
+          <t>Francisca Fadairo</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2021-2024</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Daniel Carstensen</t>
+          <t>Ameer Talha Yasser</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2021-2024</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Safwan Rashid</t>
+          <t>Yue Zhuo</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1767,7 +1767,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Francisca Fadairo</t>
+          <t>Charles Baker</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1779,7 +1779,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Ameer Talha Yasser</t>
+          <t>Andrew Shi</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1791,7 +1791,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Yue Zhuo</t>
+          <t>Ash Chinta</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1803,7 +1803,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Charles Baker</t>
+          <t>Xueyao Zheng</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1815,7 +1815,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Andrew Shi</t>
+          <t>Sergio Campos Legonia</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1827,7 +1827,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Ash Chinta</t>
+          <t>Elias Emery</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1839,7 +1839,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Xueyao Zheng</t>
+          <t>Yvonne Chen</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1851,7 +1851,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Sergio Campos Legonia</t>
+          <t>William McCall</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1863,7 +1863,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Elias Emery</t>
+          <t>Natalie Schreder</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1875,7 +1875,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Yvonne Chen</t>
+          <t>Raselas Dessalegn</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1887,7 +1887,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>William McCall</t>
+          <t>Grace Wang</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1899,55 +1899,55 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Natalie Schreder</t>
+          <t>Ansh Patel</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022-2024</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Raselas Dessalegn</t>
+          <t>Ziyan Zhu</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022-2023</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Grace Wang</t>
+          <t>Anna Mikhailova</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Ziyan Zhu</t>
+          <t>Benjamin Lehrburger</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2022-2023</t>
+          <t>2022</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Anna Mikhailova</t>
+          <t>Thomas Corrado</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1959,7 +1959,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Benjamin Lehrburger</t>
+          <t>Samuel Crombie</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1971,7 +1971,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Thomas Corrado</t>
+          <t>Alexander Marcoux</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1983,7 +1983,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Samuel Crombie</t>
+          <t>Jessna Brar</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1995,7 +1995,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Alexander Marcoux</t>
+          <t>Wenhua Liang</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2007,7 +2007,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Jessna Brar</t>
+          <t>Kevin Cao</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2019,7 +2019,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Wenhua Liang</t>
+          <t>Goutham Veeramachaneni</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2031,7 +2031,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Kevin Cao</t>
+          <t>Zachary Somma</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2043,7 +2043,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Goutham Veeramachaneni</t>
+          <t>Dawson Haddox</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2055,7 +2055,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Zachary Somma</t>
+          <t>Swestha Jain</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2067,24 +2067,24 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Dawson Haddox</t>
+          <t>Kunal Jha</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2021-2024</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Swestha Jain</t>
+          <t>Daniel Carstensen</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2021-2024</t>
         </is>
       </c>
     </row>
@@ -2103,72 +2103,72 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Tyler Chen</t>
+          <t>Aidan Adams</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2020-2022</t>
+          <t>2021</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Chris Jun</t>
+          <t>Damini Kohli</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2020-2022</t>
+          <t>2021</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Ethan Adner</t>
+          <t>Daniel Ha</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2020-2022</t>
+          <t>2021</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Aidan Adams</t>
+          <t>Tyler Chen</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2020-2022</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Damini Kohli</t>
+          <t>Chris Jun</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2020-2022</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Daniel Ha</t>
+          <t>Ethan Adner</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2020-2022</t>
         </is>
       </c>
     </row>
@@ -2235,19 +2235,19 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Tudor Muntianu</t>
+          <t>Helen Liu</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2019-2021</t>
+          <t>2020</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Helen Liu</t>
+          <t>Kelly Rutherford</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2259,7 +2259,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Kelly Rutherford</t>
+          <t>Luca Lit</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2271,7 +2271,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Luca Lit</t>
+          <t>Vivian Tran</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2283,7 +2283,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Vivian Tran</t>
+          <t>Greg Han</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2295,7 +2295,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Greg Han</t>
+          <t>Austin Zhang</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2307,7 +2307,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Austin Zhang</t>
+          <t>Chelsea Uddenberg</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2319,7 +2319,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Chelsea Uddenberg</t>
+          <t>Shane Hewitt</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2331,7 +2331,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Shane Hewitt</t>
+          <t>Chetan Palvuluri</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2343,12 +2343,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Chetan Palvuluri</t>
+          <t>Tudor Muntianu</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2019-2021</t>
         </is>
       </c>
     </row>
@@ -2427,43 +2427,43 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Madeline Lee</t>
+          <t>William Baxley</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2016-2020</t>
+          <t>2018-2019</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>William Baxley</t>
+          <t>Ann Carpenter</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2018-2019</t>
+          <t>2018</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Paxton Fitzpatrick</t>
+          <t>Seung Ju Lee</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2017-2019</t>
+          <t>2018</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Ann Carpenter</t>
+          <t>Mustafa Nasir-Moin</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2475,7 +2475,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Seung Ju Lee</t>
+          <t>Iain Sheerin</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2487,7 +2487,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Mustafa Nasir-Moin</t>
+          <t>Darya Romanova</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2499,7 +2499,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Iain Sheerin</t>
+          <t>Rachael Chacko</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2511,7 +2511,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Darya Romanova</t>
+          <t>Kirsten Soh</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2523,31 +2523,31 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Rachael Chacko</t>
+          <t>Paxton Fitzpatrick</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2017-2019</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Kirsten Soh</t>
+          <t>Stephen Satterthwaite</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2017-2018</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Stephen Satterthwaite</t>
+          <t>Bryan Bollinger</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2559,48 +2559,48 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Bryan Bollinger</t>
+          <t>Christina Lu</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2017-2018</t>
+          <t>2017</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Campbell Field</t>
+          <t>Armando Oritz</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2016-2018</t>
+          <t>2017</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Christina Lu</t>
+          <t>Madeline Lee</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2016-2020</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Armando Oritz</t>
+          <t>Campbell Field</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2016-2018</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
added SAH to people page
</commit_message>
<xml_diff>
--- a/data/people.xlsx
+++ b/data/people.xlsx
@@ -925,6 +925,11 @@
       </c>
     </row>
     <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>sam_haskel.png</t>
+        </is>
+      </c>
       <c r="B19" t="inlineStr">
         <is>
           <t>sam haskel</t>
@@ -937,7 +942,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Sam is a Quantitative Social Science and Economics double major. He is interested in how social peer influences shape beliefs and affect how people make decisions.</t>
+          <t>Sam is a double major in Quantitative Social Science and Economics, interested in how social peer influences shape beliefs and affect decision-making. He enjoys playing sports, spending time outdoors, and hanging out with friends and family.</t>
         </is>
       </c>
     </row>
@@ -996,7 +1001,6 @@
           <t>jason kang</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
           <t>undergrad</t>

</xml_diff>

<commit_message>
added AL image to people page
</commit_message>
<xml_diff>
--- a/data/people.xlsx
+++ b/data/people.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jmanning/contextlab.github.io/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DBBEC25-5C68-704C-A5DE-1475A9D4765E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9FD7DD6-0A82-9D4B-B1DD-1C4FE879587F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="35720" yWindow="7140" windowWidth="34560" windowHeight="21660" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="287">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="288">
   <si>
     <t>image</t>
   </si>
@@ -887,6 +887,9 @@
   </si>
   <si>
     <t>evan_mcdermid.png</t>
+  </si>
+  <si>
+    <t>angelyn_liu.png</t>
   </si>
 </sst>
 </file>
@@ -1487,6 +1490,9 @@
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>287</v>
+      </c>
       <c r="B13" t="s">
         <v>43</v>
       </c>

</xml_diff>

<commit_message>
Offboarded Kevin Chang to alumni
Moved Kevin Chang from active members to alumni_undergrads (2025-2026),
updated CV entry, and rebuilt people.html.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/people.xlsx
+++ b/data/people.xlsx
@@ -520,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="32.83203125" customWidth="1" min="1" max="1"/>
@@ -921,9 +921,14 @@
       </c>
     </row>
     <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>sam_haskel.png</t>
+        </is>
+      </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>kevin chang</t>
+          <t>sam haskel</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -933,19 +938,19 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>From Taipei and Boston, Kevin is a ‘29 studying Applied Math and CS. He is passionate about quantitative finance, machine learning, and health analytics. His long term goal is to develop data-driven solutions to optimize inefficiencies in the US healthcare system.</t>
+          <t>Sam is a double major in Quantitative Social Science and Economics, interested in how social peer influences shape beliefs and affect decision-making. He enjoys playing sports, spending time outdoors, and hanging out with friends and family.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>sam_haskel.png</t>
+          <t>will_lehman.png</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>sam haskel</t>
+          <t>will lehman</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -955,19 +960,19 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Sam is a double major in Quantitative Social Science and Economics, interested in how social peer influences shape beliefs and affect decision-making. He enjoys playing sports, spending time outdoors, and hanging out with friends and family.</t>
+          <t>Will is a '27 from Salt Lake City, Utah. He likes skiing, playing hockey, and working on new projects.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>will_lehman.png</t>
+          <t>theo_larson.png</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>will lehman</t>
+          <t>theo larson</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -977,19 +982,19 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Will is a '27 from Salt Lake City, Utah. He likes skiing, playing hockey, and working on new projects.</t>
+          <t>Theo is a '29 from Brooklyn, New York and a prospective major in Economics and History. In his free time, he enjoys reading, playing board games, and taking walks with his dog Sunny.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>theo_larson.png</t>
+          <t>jason_kang.png</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>theo larson</t>
+          <t>jason kang</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -999,19 +1004,19 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Theo is a '29 from Brooklyn, New York and a prospective major in Economics and History. In his free time, he enjoys reading, playing board games, and taking walks with his dog Sunny.</t>
+          <t>Jason, a member of the class of 2028, plans to major in Psychology. He enjoys games, hiking, and watching sports like basketball and tennis.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>jason_kang.png</t>
+          <t>mak_kelly.png</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>jason kang</t>
+          <t>mak kelly</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1021,19 +1026,19 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Jason, a member of the class of 2028, plans to major in Psychology. He enjoys games, hiking, and watching sports like basketball and tennis.</t>
+          <t>Mak, a '28 math and computer science major, is interested in entrepreneurship and plays rugby for Dartmouth.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>mak_kelly.png</t>
+          <t>isaac_cheon.png</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>mak kelly</t>
+          <t>isaac cheon</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1043,19 +1048,19 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Mak, a '28 math and computer science major, is interested in entrepreneurship and plays rugby for Dartmouth.</t>
+          <t>Isaac is a pre-dental student majoring in Computer Science. He enjoys playing drums and spending time outdoors.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>isaac_cheon.png</t>
+          <t>ahmad_wahab.png</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>isaac cheon</t>
+          <t>ahmad wahab</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1064,29 +1069,6 @@
         </is>
       </c>
       <c r="E24" t="inlineStr">
-        <is>
-          <t>Isaac is a pre-dental student majoring in Computer Science. He enjoys playing drums and spending time outdoors.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>ahmad_wahab.png</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>ahmad wahab</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>undergrad</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
         <is>
           <t>Ahmad, a Dartmouth '27 student, studies computer science and neuroscience, focusing on applying technology to solve real-world healthcare issues. In his free time, he enjoys rock climbing.</t>
         </is>
@@ -1474,7 +1456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D114"/>
+  <dimension ref="A1:D115"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1502,7 +1484,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Jackson C. Sandrich</t>
+          <t>Kevin Chang</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1514,7 +1496,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Luca Gandrud</t>
+          <t>Jackson C. Sandrich</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1526,7 +1508,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Annabelle Morrow</t>
+          <t>Luca Gandrud</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1538,7 +1520,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Owen Phillips</t>
+          <t>Annabelle Morrow</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1550,55 +1532,55 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Rodrigo Vega Ayllon</t>
+          <t>Owen Phillips</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025-2026</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Chelsea Joe</t>
+          <t>Rodrigo Vega Ayllon</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2024-2026</t>
+          <t>2025</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Harrison Stropkay</t>
+          <t>Chelsea Joe</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2024-2025</t>
+          <t>2024-2026</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Miel Wewerka</t>
+          <t>Harrison Stropkay</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024-2025</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Manraaj Singh</t>
+          <t>Miel Wewerka</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1610,7 +1592,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Can Kam</t>
+          <t>Manraaj Singh</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1622,7 +1604,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Rohan Goyal</t>
+          <t>Can Kam</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1634,7 +1616,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Abigayle McCusker</t>
+          <t>Rohan Goyal</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1646,7 +1628,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Torsha Chakraverty</t>
+          <t>Abigayle McCusker</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1658,7 +1640,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Chloe Terestchenko</t>
+          <t>Torsha Chakraverty</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1670,7 +1652,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Ansh Motiani</t>
+          <t>Chloe Terestchenko</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1682,7 +1664,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Kaitlyn Peng</t>
+          <t>Ansh Motiani</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1694,7 +1676,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Everett Tai</t>
+          <t>Kaitlyn Peng</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1706,7 +1688,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Andrew Cao</t>
+          <t>Everett Tai</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1718,31 +1700,31 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Jake McDermid</t>
+          <t>Andrew Cao</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2023-2025</t>
+          <t>2024</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Michael Chen</t>
+          <t>Jake McDermid</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2023-2025</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Grady Redding</t>
+          <t>Michael Chen</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1754,7 +1736,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>DJ Matusz</t>
+          <t>Grady Redding</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1766,7 +1748,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aaryan Agarwal</t>
+          <t>DJ Matusz</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1778,7 +1760,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Maura Hough</t>
+          <t>Aaryan Agarwal</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1790,7 +1772,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Emma Reeder</t>
+          <t>Maura Hough</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1802,7 +1784,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Megan Liu</t>
+          <t>Emma Reeder</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1814,7 +1796,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Mira Chiruvolu</t>
+          <t>Megan Liu</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1826,19 +1808,19 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Safwan Rashid</t>
+          <t>Mira Chiruvolu</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023-2024</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Francisca Fadairo</t>
+          <t>Safwan Rashid</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1850,7 +1832,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Ameer Talha Yasser</t>
+          <t>Francisca Fadairo</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1862,7 +1844,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Yue Zhuo</t>
+          <t>Ameer Talha Yasser</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1874,7 +1856,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Charles Baker</t>
+          <t>Yue Zhuo</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1886,7 +1868,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Andrew Shi</t>
+          <t>Charles Baker</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1898,7 +1880,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Ash Chinta</t>
+          <t>Andrew Shi</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1910,7 +1892,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Xueyao Zheng</t>
+          <t>Ash Chinta</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1922,7 +1904,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Sergio Campos Legonia</t>
+          <t>Xueyao Zheng</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1934,7 +1916,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Elias Emery</t>
+          <t>Sergio Campos Legonia</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1946,7 +1928,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Yvonne Chen</t>
+          <t>Elias Emery</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1958,7 +1940,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>William McCall</t>
+          <t>Yvonne Chen</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1970,7 +1952,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Natalie Schreder</t>
+          <t>William McCall</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1982,7 +1964,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Raselas Dessalegn</t>
+          <t>Natalie Schreder</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1994,7 +1976,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Grace Wang</t>
+          <t>Raselas Dessalegn</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2006,43 +1988,43 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Ansh Patel</t>
+          <t>Grace Wang</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2022-2024</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Ziyan Zhu</t>
+          <t>Ansh Patel</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2022-2023</t>
+          <t>2022-2024</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Anna Mikhailova</t>
+          <t>Ziyan Zhu</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022-2023</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Benjamin Lehrburger</t>
+          <t>Anna Mikhailova</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2054,7 +2036,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Thomas Corrado</t>
+          <t>Benjamin Lehrburger</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2066,7 +2048,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Samuel Crombie</t>
+          <t>Thomas Corrado</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2078,7 +2060,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Alexander Marcoux</t>
+          <t>Samuel Crombie</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2090,7 +2072,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Jessna Brar</t>
+          <t>Alexander Marcoux</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2102,7 +2084,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Wenhua Liang</t>
+          <t>Jessna Brar</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2114,7 +2096,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Kevin Cao</t>
+          <t>Wenhua Liang</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2126,7 +2108,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Goutham Veeramachaneni</t>
+          <t>Kevin Cao</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2138,7 +2120,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Zachary Somma</t>
+          <t>Goutham Veeramachaneni</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2150,7 +2132,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Dawson Haddox</t>
+          <t>Zachary Somma</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2162,7 +2144,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Swestha Jain</t>
+          <t>Dawson Haddox</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2174,19 +2156,19 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Kunal Jha</t>
+          <t>Swestha Jain</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2021-2024</t>
+          <t>2022</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Daniel Carstensen</t>
+          <t>Kunal Jha</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2198,31 +2180,31 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Brian Chiang</t>
+          <t>Daniel Carstensen</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2021-2022</t>
+          <t>2021-2024</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Aidan Adams</t>
+          <t>Brian Chiang</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021-2022</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Damini Kohli</t>
+          <t>Aidan Adams</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2234,7 +2216,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Daniel Ha</t>
+          <t>Damini Kohli</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2246,19 +2228,19 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Tyler Chen</t>
+          <t>Daniel Ha</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2020-2022</t>
+          <t>2021</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Chris Jun</t>
+          <t>Tyler Chen</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2270,7 +2252,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Ethan Adner</t>
+          <t>Chris Jun</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2282,19 +2264,19 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Darren Gu</t>
+          <t>Ethan Adner</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2020-2021</t>
+          <t>2020-2022</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Tehut Biru</t>
+          <t>Darren Gu</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2306,7 +2288,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Chris Suh</t>
+          <t>Tehut Biru</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2318,7 +2300,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Chris Long</t>
+          <t>Chris Suh</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2330,7 +2312,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Esme Chen</t>
+          <t>Chris Long</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2342,19 +2324,19 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Helen Liu</t>
+          <t>Esme Chen</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2020-2021</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Kelly Rutherford</t>
+          <t>Helen Liu</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2366,7 +2348,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Luca Lit</t>
+          <t>Kelly Rutherford</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2378,7 +2360,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Vivian Tran</t>
+          <t>Luca Lit</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2390,7 +2372,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Greg Han</t>
+          <t>Vivian Tran</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2402,7 +2384,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Austin Zhang</t>
+          <t>Greg Han</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2414,7 +2396,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Chelsea Uddenberg</t>
+          <t>Austin Zhang</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2426,7 +2408,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Shane Hewitt</t>
+          <t>Chelsea Uddenberg</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2438,7 +2420,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Chetan Palvuluri</t>
+          <t>Shane Hewitt</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2450,31 +2432,31 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Tudor Muntianu</t>
+          <t>Chetan Palvuluri</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2019-2021</t>
+          <t>2020</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Aaron Lee</t>
+          <t>Tudor Muntianu</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2019-2020</t>
+          <t>2019-2021</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Anne George</t>
+          <t>Aaron Lee</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2486,7 +2468,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Sarah Park</t>
+          <t>Anne George</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2498,7 +2480,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Shane Park</t>
+          <t>Sarah Park</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2510,7 +2492,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>William Chen</t>
+          <t>Shane Park</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2522,43 +2504,43 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Alejandro Martinez</t>
+          <t>William Chen</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2018-2020</t>
+          <t>2019-2020</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>William Baxley</t>
+          <t>Alejandro Martinez</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2018-2019</t>
+          <t>2018-2020</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Ann Carpenter</t>
+          <t>William Baxley</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2018-2019</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Seung Ju Lee</t>
+          <t>Ann Carpenter</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2570,7 +2552,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Mustafa Nasir-Moin</t>
+          <t>Seung Ju Lee</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2582,7 +2564,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Iain Sheerin</t>
+          <t>Mustafa Nasir-Moin</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2594,7 +2576,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Darya Romanova</t>
+          <t>Iain Sheerin</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2606,7 +2588,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Rachael Chacko</t>
+          <t>Darya Romanova</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2618,7 +2600,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Kirsten Soh</t>
+          <t>Rachael Chacko</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2630,31 +2612,31 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Paxton Fitzpatrick</t>
+          <t>Kirsten Soh</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2017-2019</t>
+          <t>2018</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Stephen Satterthwaite</t>
+          <t>Paxton Fitzpatrick</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2017-2018</t>
+          <t>2017-2019</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Bryan Bollinger</t>
+          <t>Stephen Satterthwaite</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2666,19 +2648,19 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Christina Lu</t>
+          <t>Bryan Bollinger</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2017-2018</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Armando Oritz</t>
+          <t>Christina Lu</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2690,43 +2672,43 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Madeline Lee</t>
+          <t>Armando Oritz</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2016-2020</t>
+          <t>2017</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Campbell Field</t>
+          <t>Madeline Lee</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2016-2018</t>
+          <t>2016-2020</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Wei Liang Samuel Ching</t>
+          <t>Campbell Field</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2016-2017</t>
+          <t>2016-2018</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Marisol Tracy</t>
+          <t>Wei Liang Samuel Ching</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2738,7 +2720,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Allison Frantz</t>
+          <t>Marisol Tracy</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2750,7 +2732,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Aamuktha Porika</t>
+          <t>Allison Frantz</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2762,19 +2744,19 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Jake Rost</t>
+          <t>Aamuktha Porika</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>2016-2017</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Clara Silvanic</t>
+          <t>Jake Rost</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -2786,7 +2768,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Aman Agarwal</t>
+          <t>Clara Silvanic</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -2798,7 +2780,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Joseph Finkelstein</t>
+          <t>Aman Agarwal</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -2810,7 +2792,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Sheherzad Mohydin</t>
+          <t>Joseph Finkelstein</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -2822,7 +2804,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Peter Tran</t>
+          <t>Sheherzad Mohydin</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -2834,7 +2816,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Gal Perlman</t>
+          <t>Peter Tran</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -2846,10 +2828,22 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
+          <t>Gal Perlman</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
           <t>Jessica Tin</t>
         </is>
       </c>
-      <c r="B114" t="inlineStr">
+      <c r="B115" t="inlineStr">
         <is>
           <t>2016</t>
         </is>

</xml_diff>

<commit_message>
Offboarded Jacob Bacus, Andrew Richardson, and Evan McDermid
Moved all three from active members to alumni_undergrads, updated CV
entries, and rebuilt people.html.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/people.xlsx
+++ b/data/people.xlsx
@@ -520,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="32.83203125" customWidth="1" min="1" max="1"/>
@@ -703,12 +703,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>jacob_bacus.png</t>
+          <t>aidan_miller.png</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>jacob bacus</t>
+          <t>aidan miller</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -718,19 +718,19 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Jacob is a member of the class of 2027 from Kansas City, Missouri studying Computer Science and Middle Eastern Studies. Jacob's work in the lab focuses on using machine learning and deep learning models to understand mental health. He is also interested in how cognitive and mental function relate to one another.</t>
+          <t>Aidan is a pre-med student at Dartmouth College, majoring in Biology, minor in Spanish, and graduating in 2028. He joined the Contextual Dynamics Lab in fall 2025, where his interests center on advanced learning and memory techniques, including the method of loci and PAO systems.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>aidan_miller.png</t>
+          <t>alexandra_wingo.png</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>aidan miller</t>
+          <t>alexandra wingo</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -740,19 +740,19 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Aidan is a pre-med student at Dartmouth College, majoring in Biology, minor in Spanish, and graduating in 2028. He joined the Contextual Dynamics Lab in fall 2025, where his interests center on advanced learning and memory techniques, including the method of loci and PAO systems.</t>
+          <t>Alexandra is interested in education technology and brings to the lab her extensive computer science experience. She is especially interested in helping students with learning differences, and in developing brain-based learning tools.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>alexandra_wingo.png</t>
+          <t>alishba_tahir.png</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>alexandra wingo</t>
+          <t>alishba tahir</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -762,19 +762,19 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Alexandra is interested in education technology and brings to the lab her extensive computer science experience. She is especially interested in helping students with learning differences, and in developing brain-based learning tools.</t>
+          <t>Alishba is a visiting research assistant interested in the intersection of memory, narrative processing, and the mechanisms behind forgetting what to forget. She holds an undergraduate degree in Biology from LUMS and has previously worked on fMRI-based disease analysis. At the CDL, she is exploring how recall and prediction shape memory dynamics over time using naturalistic stimuli.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>alishba_tahir.png</t>
+          <t>angelyn_liu.png</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>alishba tahir</t>
+          <t>angelyn liu</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -784,19 +784,19 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Alishba is a visiting research assistant interested in the intersection of memory, narrative processing, and the mechanisms behind forgetting what to forget. She holds an undergraduate degree in Biology from LUMS and has previously worked on fMRI-based disease analysis. At the CDL, she is exploring how recall and prediction shape memory dynamics over time using naturalistic stimuli.</t>
+          <t>Angelyn is a member of the class of 2028 from the Bay Area, CA, planning on majoring in cognitive science. In her free time, she enjoys singing, reading, puzzle games, and creative writing.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>andrew_richardson.png</t>
+          <t>azaire_andre.png</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>andrew richardson</t>
+          <t>azaire andre</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -806,19 +806,19 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Andrew is a Mathematics and Economics double major from Minneapolis, MN. Outside of academics, he enjoys playing tennis and soccer.</t>
+          <t>Azaire is a Dartmouth student studying mathematics and anthropology, with interests in health equity, education, and community leadership. She enjoys swimming and cheering, and is actively involved in campus organizations that support mentorship and inclusion.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>angelyn_liu.png</t>
+          <t>ben_hanson.png</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>angelyn liu</t>
+          <t>ben hanson</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -828,19 +828,19 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Angelyn is a member of the class of 2028 from the Bay Area, CA, planning on majoring in cognitive science. In her free time, she enjoys singing, reading, puzzle games, and creative writing.</t>
+          <t>Ben is a member of the class of 2027 studying PPE and human-centered design. Outside of school, he enjoy skiing, surfing, and coffee.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>azaire_andre.png</t>
+          <t>ellie_mattox.png</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>azaire andre</t>
+          <t>ellie mattox</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -850,19 +850,19 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Azaire is a Dartmouth student studying mathematics and anthropology, with interests in health equity, education, and community leadership. She enjoys swimming and cheering, and is actively involved in campus organizations that support mentorship and inclusion.</t>
+          <t>Ellie is a member of the class of 2027 from Austin, TX and is majoring in neuroscience with a minor in human-centered design. Outside of the lab she enjoys playing volleyball on Dartmouth's Varsity team, spending time outside, and hanging out with friends.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ben_hanson.png</t>
+          <t>sam_haskel.png</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ben hanson</t>
+          <t>sam haskel</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -872,19 +872,19 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Ben is a member of the class of 2027 studying PPE and human-centered design. Outside of school, he enjoy skiing, surfing, and coffee.</t>
+          <t>Sam is a double major in Quantitative Social Science and Economics, interested in how social peer influences shape beliefs and affect decision-making. He enjoys playing sports, spending time outdoors, and hanging out with friends and family.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ellie_mattox.png</t>
+          <t>will_lehman.png</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ellie mattox</t>
+          <t>will lehman</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -894,19 +894,19 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Ellie is a member of the class of 2027 from Austin, TX and is majoring in neuroscience with a minor in human-centered design. Outside of the lab she enjoys playing volleyball on Dartmouth's Varsity team, spending time outside, and hanging out with friends.</t>
+          <t>Will is a '27 from Salt Lake City, Utah. He likes skiing, playing hockey, and working on new projects.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>evan_mcdermid.png</t>
+          <t>theo_larson.png</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>evan mcdermid</t>
+          <t>theo larson</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -916,19 +916,19 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Evan is a Mathematics major and Computer Science minor. He is interested in algorithmic trading, algorithmic problem solving, and building models of financial market dynamics.</t>
+          <t>Theo is a '29 from Brooklyn, New York and a prospective major in Economics and History. In his free time, he enjoys reading, playing board games, and taking walks with his dog Sunny.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>sam_haskel.png</t>
+          <t>jason_kang.png</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>sam haskel</t>
+          <t>jason kang</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -938,19 +938,19 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Sam is a double major in Quantitative Social Science and Economics, interested in how social peer influences shape beliefs and affect decision-making. He enjoys playing sports, spending time outdoors, and hanging out with friends and family.</t>
+          <t>Jason, a member of the class of 2028, plans to major in Psychology. He enjoys games, hiking, and watching sports like basketball and tennis.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>will_lehman.png</t>
+          <t>mak_kelly.png</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>will lehman</t>
+          <t>mak kelly</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -960,19 +960,19 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Will is a '27 from Salt Lake City, Utah. He likes skiing, playing hockey, and working on new projects.</t>
+          <t>Mak, a '28 math and computer science major, is interested in entrepreneurship and plays rugby for Dartmouth.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>theo_larson.png</t>
+          <t>isaac_cheon.png</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>theo larson</t>
+          <t>isaac cheon</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -982,19 +982,19 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Theo is a '29 from Brooklyn, New York and a prospective major in Economics and History. In his free time, he enjoys reading, playing board games, and taking walks with his dog Sunny.</t>
+          <t>Isaac is a pre-dental student majoring in Computer Science. He enjoys playing drums and spending time outdoors.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>jason_kang.png</t>
+          <t>ahmad_wahab.png</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>jason kang</t>
+          <t>ahmad wahab</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1003,72 +1003,6 @@
         </is>
       </c>
       <c r="E21" t="inlineStr">
-        <is>
-          <t>Jason, a member of the class of 2028, plans to major in Psychology. He enjoys games, hiking, and watching sports like basketball and tennis.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>mak_kelly.png</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>mak kelly</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>undergrad</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Mak, a '28 math and computer science major, is interested in entrepreneurship and plays rugby for Dartmouth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>isaac_cheon.png</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>isaac cheon</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>undergrad</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Isaac is a pre-dental student majoring in Computer Science. He enjoys playing drums and spending time outdoors.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>ahmad_wahab.png</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>ahmad wahab</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>undergrad</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
         <is>
           <t>Ahmad, a Dartmouth '27 student, studies computer science and neuroscience, focusing on applying technology to solve real-world healthcare issues. In his free time, he enjoys rock climbing.</t>
         </is>
@@ -1456,7 +1390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D115"/>
+  <dimension ref="A1:D118"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1484,7 +1418,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Kevin Chang</t>
+          <t>Evan Mcdermid</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1496,7 +1430,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Jackson C. Sandrich</t>
+          <t>Andrew Richardson</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1508,19 +1442,19 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Luca Gandrud</t>
+          <t>Jacob Bacus</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2024-2026</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Annabelle Morrow</t>
+          <t>Kevin Chang</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1532,7 +1466,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Owen Phillips</t>
+          <t>Jackson C. Sandrich</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1544,79 +1478,79 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Rodrigo Vega Ayllon</t>
+          <t>Luca Gandrud</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025-2026</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Chelsea Joe</t>
+          <t>Annabelle Morrow</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2024-2026</t>
+          <t>2025-2026</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Harrison Stropkay</t>
+          <t>Owen Phillips</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2024-2025</t>
+          <t>2025-2026</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Miel Wewerka</t>
+          <t>Rodrigo Vega Ayllon</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2025</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Manraaj Singh</t>
+          <t>Chelsea Joe</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024-2026</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Can Kam</t>
+          <t>Harrison Stropkay</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024-2025</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Rohan Goyal</t>
+          <t>Miel Wewerka</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1628,7 +1562,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Abigayle McCusker</t>
+          <t>Manraaj Singh</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1640,7 +1574,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Torsha Chakraverty</t>
+          <t>Can Kam</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1652,7 +1586,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Chloe Terestchenko</t>
+          <t>Rohan Goyal</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1664,7 +1598,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Ansh Motiani</t>
+          <t>Abigayle McCusker</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1676,7 +1610,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Kaitlyn Peng</t>
+          <t>Torsha Chakraverty</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1688,7 +1622,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Everett Tai</t>
+          <t>Chloe Terestchenko</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1700,7 +1634,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Andrew Cao</t>
+          <t>Ansh Motiani</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1712,55 +1646,55 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Jake McDermid</t>
+          <t>Kaitlyn Peng</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2023-2025</t>
+          <t>2024</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Michael Chen</t>
+          <t>Everett Tai</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2024</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Grady Redding</t>
+          <t>Andrew Cao</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2024</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>DJ Matusz</t>
+          <t>Jake McDermid</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2023-2025</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Aaryan Agarwal</t>
+          <t>Michael Chen</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1772,7 +1706,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Maura Hough</t>
+          <t>Grady Redding</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1784,7 +1718,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Emma Reeder</t>
+          <t>DJ Matusz</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1796,7 +1730,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Megan Liu</t>
+          <t>Aaryan Agarwal</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1808,7 +1742,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Mira Chiruvolu</t>
+          <t>Maura Hough</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1820,43 +1754,43 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Safwan Rashid</t>
+          <t>Emma Reeder</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023-2024</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Francisca Fadairo</t>
+          <t>Megan Liu</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023-2024</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Ameer Talha Yasser</t>
+          <t>Mira Chiruvolu</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023-2024</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Yue Zhuo</t>
+          <t>Safwan Rashid</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1868,7 +1802,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Charles Baker</t>
+          <t>Francisca Fadairo</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1880,7 +1814,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Andrew Shi</t>
+          <t>Ameer Talha Yasser</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1892,7 +1826,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Ash Chinta</t>
+          <t>Yue Zhuo</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1904,7 +1838,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Xueyao Zheng</t>
+          <t>Charles Baker</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1916,7 +1850,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Sergio Campos Legonia</t>
+          <t>Andrew Shi</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1928,7 +1862,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Elias Emery</t>
+          <t>Ash Chinta</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1940,7 +1874,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Yvonne Chen</t>
+          <t>Xueyao Zheng</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1952,7 +1886,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>William McCall</t>
+          <t>Sergio Campos Legonia</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1964,7 +1898,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Natalie Schreder</t>
+          <t>Elias Emery</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1976,7 +1910,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Raselas Dessalegn</t>
+          <t>Yvonne Chen</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1988,7 +1922,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Grace Wang</t>
+          <t>William McCall</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2000,67 +1934,67 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Ansh Patel</t>
+          <t>Natalie Schreder</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2022-2024</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Ziyan Zhu</t>
+          <t>Raselas Dessalegn</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2022-2023</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Anna Mikhailova</t>
+          <t>Grace Wang</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Benjamin Lehrburger</t>
+          <t>Ansh Patel</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022-2024</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Thomas Corrado</t>
+          <t>Ziyan Zhu</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022-2023</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Samuel Crombie</t>
+          <t>Anna Mikhailova</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2072,7 +2006,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Alexander Marcoux</t>
+          <t>Benjamin Lehrburger</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2084,7 +2018,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Jessna Brar</t>
+          <t>Thomas Corrado</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2096,7 +2030,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Wenhua Liang</t>
+          <t>Samuel Crombie</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2108,7 +2042,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Kevin Cao</t>
+          <t>Alexander Marcoux</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2120,7 +2054,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Goutham Veeramachaneni</t>
+          <t>Jessna Brar</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2132,7 +2066,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Zachary Somma</t>
+          <t>Wenhua Liang</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2144,7 +2078,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Dawson Haddox</t>
+          <t>Kevin Cao</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2156,7 +2090,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Swestha Jain</t>
+          <t>Goutham Veeramachaneni</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2168,151 +2102,151 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Kunal Jha</t>
+          <t>Zachary Somma</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2021-2024</t>
+          <t>2022</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Daniel Carstensen</t>
+          <t>Dawson Haddox</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2021-2024</t>
+          <t>2022</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Brian Chiang</t>
+          <t>Swestha Jain</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2021-2022</t>
+          <t>2022</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Aidan Adams</t>
+          <t>Kunal Jha</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021-2024</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Damini Kohli</t>
+          <t>Daniel Carstensen</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021-2024</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Daniel Ha</t>
+          <t>Brian Chiang</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021-2022</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Tyler Chen</t>
+          <t>Aidan Adams</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2020-2022</t>
+          <t>2021</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Chris Jun</t>
+          <t>Damini Kohli</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2020-2022</t>
+          <t>2021</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Ethan Adner</t>
+          <t>Daniel Ha</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2020-2022</t>
+          <t>2021</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Darren Gu</t>
+          <t>Tyler Chen</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2020-2021</t>
+          <t>2020-2022</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Tehut Biru</t>
+          <t>Chris Jun</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2020-2021</t>
+          <t>2020-2022</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Chris Suh</t>
+          <t>Ethan Adner</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2020-2021</t>
+          <t>2020-2022</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Chris Long</t>
+          <t>Darren Gu</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2324,7 +2258,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Esme Chen</t>
+          <t>Tehut Biru</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2336,43 +2270,43 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Helen Liu</t>
+          <t>Chris Suh</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2020-2021</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Kelly Rutherford</t>
+          <t>Chris Long</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2020-2021</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Luca Lit</t>
+          <t>Esme Chen</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2020-2021</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Vivian Tran</t>
+          <t>Helen Liu</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2384,7 +2318,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Greg Han</t>
+          <t>Kelly Rutherford</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2396,7 +2330,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Austin Zhang</t>
+          <t>Luca Lit</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2408,7 +2342,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Chelsea Uddenberg</t>
+          <t>Vivian Tran</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2420,7 +2354,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Shane Hewitt</t>
+          <t>Greg Han</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2432,7 +2366,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Chetan Palvuluri</t>
+          <t>Austin Zhang</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2444,55 +2378,55 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Tudor Muntianu</t>
+          <t>Chelsea Uddenberg</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2019-2021</t>
+          <t>2020</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Aaron Lee</t>
+          <t>Shane Hewitt</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2019-2020</t>
+          <t>2020</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Anne George</t>
+          <t>Chetan Palvuluri</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2019-2020</t>
+          <t>2020</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Sarah Park</t>
+          <t>Tudor Muntianu</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2019-2020</t>
+          <t>2019-2021</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Shane Park</t>
+          <t>Aaron Lee</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2504,7 +2438,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>William Chen</t>
+          <t>Anne George</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2516,67 +2450,67 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Alejandro Martinez</t>
+          <t>Sarah Park</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2018-2020</t>
+          <t>2019-2020</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>William Baxley</t>
+          <t>Shane Park</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2018-2019</t>
+          <t>2019-2020</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Ann Carpenter</t>
+          <t>William Chen</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2019-2020</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Seung Ju Lee</t>
+          <t>Alejandro Martinez</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2018-2020</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Mustafa Nasir-Moin</t>
+          <t>William Baxley</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2018-2019</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Iain Sheerin</t>
+          <t>Ann Carpenter</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2588,7 +2522,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Darya Romanova</t>
+          <t>Seung Ju Lee</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2600,7 +2534,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Rachael Chacko</t>
+          <t>Mustafa Nasir-Moin</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2612,7 +2546,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Kirsten Soh</t>
+          <t>Iain Sheerin</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2624,127 +2558,127 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Paxton Fitzpatrick</t>
+          <t>Darya Romanova</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2017-2019</t>
+          <t>2018</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Stephen Satterthwaite</t>
+          <t>Rachael Chacko</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2017-2018</t>
+          <t>2018</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Bryan Bollinger</t>
+          <t>Kirsten Soh</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2017-2018</t>
+          <t>2018</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Christina Lu</t>
+          <t>Paxton Fitzpatrick</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2017-2019</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Armando Oritz</t>
+          <t>Stephen Satterthwaite</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2017-2018</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Madeline Lee</t>
+          <t>Bryan Bollinger</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2016-2020</t>
+          <t>2017-2018</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Campbell Field</t>
+          <t>Christina Lu</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2016-2018</t>
+          <t>2017</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Wei Liang Samuel Ching</t>
+          <t>Armando Oritz</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2016-2017</t>
+          <t>2017</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Marisol Tracy</t>
+          <t>Madeline Lee</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2016-2017</t>
+          <t>2016-2020</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Allison Frantz</t>
+          <t>Campbell Field</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2016-2017</t>
+          <t>2016-2018</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Aamuktha Porika</t>
+          <t>Wei Liang Samuel Ching</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -2756,43 +2690,43 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Jake Rost</t>
+          <t>Marisol Tracy</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>2016-2017</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Clara Silvanic</t>
+          <t>Allison Frantz</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>2016-2017</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Aman Agarwal</t>
+          <t>Aamuktha Porika</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>2016-2017</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Joseph Finkelstein</t>
+          <t>Jake Rost</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -2804,7 +2738,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Sheherzad Mohydin</t>
+          <t>Clara Silvanic</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -2816,7 +2750,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Peter Tran</t>
+          <t>Aman Agarwal</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -2828,7 +2762,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Gal Perlman</t>
+          <t>Joseph Finkelstein</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -2840,10 +2774,46 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
+          <t>Sheherzad Mohydin</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Peter Tran</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Gal Perlman</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
           <t>Jessica Tin</t>
         </is>
       </c>
-      <c r="B115" t="inlineStr">
+      <c r="B118" t="inlineStr">
         <is>
           <t>2016</t>
         </is>

</xml_diff>

<commit_message>
Reconcile people data and onboard Andy Kim
Data fixes from reconciliation dry-run:
- Fixed spelling: Aaryan Agarwal → Aaryan Agrawal in people.xlsx
- Fixed name: Maura F. Hough → Maura Hough in lab-manual
- Fixed name: Francisca O. Fadairo → Francisca Fadairo in lab-manual
- Offboarded Maura Hough (2023) to alumni in lab-manual

Added to alumni_undergrads in people.xlsx (flagged by reconciliation):
- Matthew Givens (2024-2025), Keene Dampal (2025), Jaysen Quan (2025)
- Molly McQuoid (2022), Joy Maina (2025), Emmy Thornton (2025)
- Moved Matt/Keene/Jaysen/Maura to alumni in lab-manual
- Added Joy/Emmy to lab-manual alumni
- Closed CV entries for Joy/Emmy

Onboarded Andy Kim (Hye-Sung Kim) as undergrad:
- Added to people.xlsx, JRM_CV.tex, lab-manual, Google calendars

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/people.xlsx
+++ b/data/people.xlsx
@@ -520,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="32.83203125" customWidth="1" min="1" max="1"/>
@@ -1005,6 +1005,29 @@
       <c r="E21" t="inlineStr">
         <is>
           <t>Ahmad, a Dartmouth '27 student, studies computer science and neuroscience, focusing on applying technology to solve real-world healthcare issues. In his free time, he enjoys rock climbing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>andy_kim.png</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>andy kim</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>undergrad</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Andy is a prospective QSS major from Seoul, South Korea. He has many academic interests involving decision-making, learning, neurodivergence, the market, and theatre. Outside of classes he works as a Tech for Collis and dances in his hip-hop dance group Street Soul.</t>
         </is>
       </c>
     </row>
@@ -1390,7 +1413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D118"/>
+  <dimension ref="A1:D124"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1730,7 +1753,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Aaryan Agarwal</t>
+          <t>Aaryan Agrawal</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2816,6 +2839,78 @@
       <c r="B118" t="inlineStr">
         <is>
           <t>2016</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Matthew Givens</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>2024-2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Keene Dampal</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Jaysen Quan</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Molly McQuoid</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Joy Maina</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Emmy Thornton</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Onboard Colson Duncan, update README with sync docs
- Onboarded Colson Duncan as undergrad (people.xlsx, CV, lab-manual,
  GitHub, Google calendars). No photo yet.
- Removed duplicate Colson entry in lab-manual (kept 2025 start year)
- Updated README.md: added lab-manual update to onboard/offboard docs,
  added reconciliation section, added submodule init to build docs
- Reconciliation now shows 0 flagged items (down from 18)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/people.xlsx
+++ b/data/people.xlsx
@@ -520,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="32.83203125" customWidth="1" min="1" max="1"/>
@@ -1027,6 +1027,23 @@
       <c r="E22" t="inlineStr">
         <is>
           <t>Andy is a prospective QSS major from Seoul, South Korea. He has many academic interests involving decision-making, learning, neurodivergence, the market, and theatre. Outside of classes he works as a Tech for Collis and dances in his hip-hop dance group Street Soul.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>colson duncan</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>undergrad</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Colson is a '27 studying Neuroscience and Biological Sciences from Los Angeles. He enjoys playing tennis, climbing and playing the guitar.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Colson Duncan's photo with hand-drawn border
Processed colson_duncan.jpg with face detection and border, updated
people.xlsx image reference, rebuilt people.html.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/people.xlsx
+++ b/data/people.xlsx
@@ -520,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="32.83203125" customWidth="1" min="1" max="1"/>
@@ -1031,6 +1031,11 @@
       </c>
     </row>
     <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>colson_duncan.png</t>
+        </is>
+      </c>
       <c r="B23" t="inlineStr">
         <is>
           <t>colson duncan</t>

</xml_diff>

<commit_message>
Onboard Miles McDonald as undergrad
Added to people.xlsx, JRM_CV.tex, lab-manual. Photo processed with
face detection and hand-drawn border. GitHub invited, calendars shared.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/people.xlsx
+++ b/data/people.xlsx
@@ -520,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="32.83203125" customWidth="1" min="1" max="1"/>
@@ -1049,6 +1049,28 @@
       <c r="E23" t="inlineStr">
         <is>
           <t>Colson is a '27 studying Neuroscience and Biological Sciences from Los Angeles. He enjoys playing tennis, climbing and playing the guitar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>miles_mcdonald.png</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>miles mcdonald</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>undergrad</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Interested in neurodivergence within inner monologues and BCIs. Excited to gain experience taking data through analysis to application.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Onboard five new undergrads (Malique, Phoom, Katherina, Abe, Martin)
- Add members to people.xlsx, CV, and lab-manual (via onboard script)
- LLM-rewritten bios (with light polish for consistent third-person style)
- Add third-person rule to onboard_member.py LLM prompt to prevent
  future first-person bios slipping through
- Remove duplicate Phoom entry from CV caused by quote-style mismatch
  during re-onboarding

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/people.xlsx
+++ b/data/people.xlsx
@@ -520,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="32.83203125" customWidth="1" min="1" max="1"/>
@@ -1071,6 +1071,116 @@
       <c r="E24" t="inlineStr">
         <is>
           <t>Miles is interested in neurodivergence within inner monologues and brain-computer interfaces. He is excited to gain experience taking data through analysis to application.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>malique_auguste.png</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>malique auguste</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>https://malique-auguste.github.io/</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>undergrad</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Malique is a double major in Applied Mathematics and Government, focusing on the quantitative tools used to investigate political and social issues. He is excited to advance the understanding of human cognition by exploring the parallels between financial markets and neural dynamics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>pattapol_sirimangklanurak.png</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>pattapol "phoom" sirimangklanurak</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>undergrad</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Phoom is a member of the class of 2028 from Chiang Mai, Thailand, studying Math and QSS. Outside of class, he is passionate about photography, Magic: The Gathering, cultural organizations on campus, and good food.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>katherina_cohen.png</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>katherina cohen</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>undergrad</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Katherina is a Government and Cognitive Science major from Buenos Aires with a strong passion for Studio Art.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>abe_lobsenz.png</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>abe lobsenz</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>undergrad</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Abe is a prospective mathematics major from Connecticut with interests in both pure and applied math. He enjoys biking, powerlifting, and hiking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>martin palencia-gomez</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>undergrad</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Martin is a sophomore at Dartmouth College studying Computer Science and Economics, with a focus on the intersection of technology and healthcare. He co-founded Acesso, a startup reimagining how patients navigate health insurance, and pursues research in financial modeling, applied machine learning, and healthcare systems.</t>
         </is>
       </c>
     </row>

</xml_diff>